<commit_message>
arccos update 2026-06-06, 1 rounds
</commit_message>
<xml_diff>
--- a/arccos_sg_baseline.xlsx
+++ b/arccos_sg_baseline.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>2026-06-06 23:33 UTC</t>
+          <t>2026-06-06 23:53 UTC</t>
         </is>
       </c>
     </row>
@@ -10670,7 +10670,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Date pulled: 2026-06-06 23:33 UTC  |  Rounds: 1  Shots: 95</t>
+          <t>Date pulled: 2026-06-06 23:53 UTC  |  Rounds: 1  Shots: 95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
arccos update 2026-06-07, 1 rounds
</commit_message>
<xml_diff>
--- a/arccos_sg_baseline.xlsx
+++ b/arccos_sg_baseline.xlsx
@@ -857,24 +857,12 @@
       <c r="AN2" t="n">
         <v>-3.82</v>
       </c>
-      <c r="AO2" t="n">
-        <v>-20.4148</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>-7.49223</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>-30</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>-30</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>-4.95085</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>-10.2852</v>
-      </c>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8178,16 +8166,8 @@
           <t>Driver</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Cobra</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DS-ADAPT LS</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>262.8</v>
       </c>
@@ -8228,16 +8208,8 @@
           <t>Wood</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Cobra</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DS-ADAPT</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>203.7</v>
       </c>
@@ -8260,24 +8232,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5 Wood</t>
+          <t>club3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wood</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Cobra</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DS-ADAPT</t>
-        </is>
-      </c>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>184</v>
       </c>
@@ -8306,16 +8270,8 @@
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Cobra</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DS-ADAPT</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>172.9</v>
       </c>
@@ -8344,16 +8300,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>155.8</v>
       </c>
@@ -8400,16 +8348,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>143.7</v>
       </c>
@@ -8440,16 +8380,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>133.6</v>
       </c>
@@ -8482,16 +8414,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>126.2</v>
       </c>
@@ -8536,16 +8460,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>122</v>
       </c>
@@ -8578,16 +8494,8 @@
           <t>Iron</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Srixon</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ZX7 Mk II</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>108.1</v>
       </c>
@@ -8628,16 +8536,8 @@
           <t>Wedge</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Cleveland</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>RTX 6 ZipCore</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>100.3</v>
       </c>
@@ -8682,16 +8582,8 @@
           <t>Wedge</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cleveland</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>RTX 6 ZipCore</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>86.8</v>
       </c>
@@ -8720,16 +8612,8 @@
           <t>Wedge</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cleveland</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>RTX 6 ZipCore</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>80.7</v>
       </c>
@@ -8770,7 +8654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8819,29 +8703,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>27924130</v>
-      </c>
-      <c r="B2" t="n">
-        <v>-20.4148</v>
-      </c>
-      <c r="C2" t="n">
-        <v>-7.49223</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-30</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-30</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-4.95085</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-10.2852</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8853,7 +8714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B144"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -8884,9 +8745,6 @@
           <t>SG total</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>-23.7</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8894,9 +8752,6 @@
           <t>SG driving</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>-1.2</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8904,9 +8759,6 @@
           <t>SG approach</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>-14.6</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8914,9 +8766,6 @@
           <t>SG short</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>-6.1</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8924,9 +8773,6 @@
           <t>SG putting</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>-1.8</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -8945,9 +8791,6 @@
           <t>fairway_pct</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>64.3</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8955,9 +8798,6 @@
           <t>gir_pct</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>27.8</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8965,9 +8805,6 @@
           <t>scramble_chip_save_pct</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8975,9 +8812,6 @@
           <t>chip_down_pct</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>11.1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8985,9 +8819,6 @@
           <t>chip_error_rate</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>18.2</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8995,9 +8826,6 @@
           <t>sand_save_pct</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9005,9 +8833,6 @@
           <t>three_putt_pct</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>16.7</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9015,9 +8840,6 @@
           <t>one_putt_pct</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>5.6</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9025,9 +8847,6 @@
           <t>putts_per_round</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -9050,1206 +8869,36 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>drive.noOfFairWaysHit</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>9</v>
+          <t>-- approach --</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>drive.noOfFairWaysRight</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0</v>
+          <t>-- chip --</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>drive.noOfFairWaysLeft</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>5</v>
+          <t>-- sand --</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>drive.noOfFairwayAttempts</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>14</v>
+          <t>-- putt --</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>drive.noOfPlusOnePenalties</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>drive.noOfRecoveryShotsHit</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>drive.noOfPlusTwoPenalties</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>drive.noOfTimesRecoveryRequired</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>drive.totalDistance</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>3035.27</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>drive.maxDistance</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>247.29</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>drive.noOfDriveShotsNotIgnored</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>drive.noOfDriveShots</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>drive.deltaDistance</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>28.86</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>drive.noOfGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>drive.noOfShort</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>drive.noOfRecoveryShots</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>drive.noOfRecoveryShotsNotIgnored</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>drive.totalDistanceRecoveryShots</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>64.45999999999999</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>drive.maxDistanceRecoveryShots</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>35.59</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>drive.deltaDistanceRecoveryShots</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>3.36</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>drive.driveHcp</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>-7.49</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>drive.expectedDistance</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>drive.expectedDistanceRangeLow</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>drive.expectedDistanceRangeHigh</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>-- approach --</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>approach.noOfPlusOnePenalties</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>approach.noOfShotsInSand</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>approach.noOfPlusTwoPenalties</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>approach.noOfGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>approach.noOfGreens</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>approach.noOfHoles</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>approach.noOfGreensHit</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>approach.noOfRight</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>approach.noOfLong</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>approach.noOfLeft</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>approach.noOfShort</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>approach.noOfApproachShots</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>approach.noOfStrokesToGetDown</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>approach.totalDistanceToPin</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>816.3099999999999</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>approach.totalDistanceToPinOnGreensHit</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>115.97</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>approach.totalDistanceToPinOnGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>73.01000000000001</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>approach.noOfLayUpShots</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>approach.approachHcp</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>-- chip --</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>chip.noOfPlusOnePenalties</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>chip.noOfErrors</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>chip.noOfPlusTwoPenalties</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>chip.noOfZeroPutts</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>chip.noOfOnePutts</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>chip.noOfTwoPutts</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>chip.noOfThreePlusPutts</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>chip.noOfChipDownChances</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>chip.noOfChipDownSuccesses</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>chip.noOfChipSaveChances</t>
-        </is>
-      </c>
-      <c r="B76" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>chip.noOfChipSaveSuccesses</t>
-        </is>
-      </c>
-      <c r="B77" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>chip.noOfChipShots</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>chip.noOfStrokesToGetDown</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPin</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>101.19</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPinOnChipDownChances</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>79.17</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPinOnChipSaveChances</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>65.29000000000001</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPinOnChipDownSuccess</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>1.83</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPinOnChipSaveSuccesses</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>chip.totalDistanceToPinOnGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>chip.noOfGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>chip.noOfRight</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>chip.noOfLong</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>chip.noOfLeft</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>chip.noOfShort</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>chip.chipHcp</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>-- sand --</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>sand.noOfPlusOnePenalties</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>sand.noOfErrors</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>sand.noOfPlusTwoPenalties</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>sand.noOfZeroPutts</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>sand.noOfOnePutts</t>
-        </is>
-      </c>
-      <c r="B97" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>sand.noOfTwoPutts</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>sand.noOfThreePlusPutts</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>sand.noOfSandDownChances</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>sand.noOfSandDownSuccesses</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>sand.noOfSandSaveChances</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>sand.noOfSandSaveSuccesses</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>sand.noOfSandShots</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>sand.noOfStrokesToGetDown</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPin</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>16.61</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPinOnSandSaveChances</t>
-        </is>
-      </c>
-      <c r="B107" t="n">
-        <v>16.61</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPinOnSandDownChances</t>
-        </is>
-      </c>
-      <c r="B108" t="n">
-        <v>16.61</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPinOnSandDownSuccesses</t>
-        </is>
-      </c>
-      <c r="B109" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPinOnSandSaveSuccesses</t>
-        </is>
-      </c>
-      <c r="B110" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>sand.totalDistanceToPinOnGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B111" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>sand.noOfGreensHitInRegulation</t>
-        </is>
-      </c>
-      <c r="B112" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>sand.noOfRight</t>
-        </is>
-      </c>
-      <c r="B113" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>sand.noOfLong</t>
-        </is>
-      </c>
-      <c r="B114" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>sand.noOfLeft</t>
-        </is>
-      </c>
-      <c r="B115" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>sand.noOfShort</t>
-        </is>
-      </c>
-      <c r="B116" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>sand.sandHcp</t>
-        </is>
-      </c>
-      <c r="B117" t="n">
-        <v>-4.95</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>-- putt --</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>putt.zeroPutts</t>
-        </is>
-      </c>
-      <c r="B119" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>putt.onePutts</t>
-        </is>
-      </c>
-      <c r="B120" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>putt.twoPutts</t>
-        </is>
-      </c>
-      <c r="B121" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>putt.threePlusPutts</t>
-        </is>
-      </c>
-      <c r="B122" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>putt.totalPutts</t>
-        </is>
-      </c>
-      <c r="B123" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>putt.noOfHoles</t>
-        </is>
-      </c>
-      <c r="B124" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>putt.noOfPuttsAfterGir</t>
-        </is>
-      </c>
-      <c r="B125" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>putt.noOfGirsHit</t>
-        </is>
-      </c>
-      <c r="B126" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>putt.noOfPlusOnePenalites</t>
-        </is>
-      </c>
-      <c r="B127" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>putt.noOfPlusTwoPenalites</t>
-        </is>
-      </c>
-      <c r="B128" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>putt.strokesGained</t>
-        </is>
-      </c>
-      <c r="B129" t="n">
-        <v>-3.1</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>putt.puttHcp</t>
-        </is>
-      </c>
-      <c r="B130" t="n">
-        <v>-10.29</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
           <t>-- overall --</t>
         </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>overall.noOfEagles</t>
-        </is>
-      </c>
-      <c r="B132" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>overall.noOfBirdies</t>
-        </is>
-      </c>
-      <c r="B133" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>overall.noOfPars</t>
-        </is>
-      </c>
-      <c r="B134" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>overall.noOfBogeys</t>
-        </is>
-      </c>
-      <c r="B135" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>overall.noOfDoubleBogeys</t>
-        </is>
-      </c>
-      <c r="B136" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>overall.noOfParThree</t>
-        </is>
-      </c>
-      <c r="B137" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>overall.parThreeTotalStrokes</t>
-        </is>
-      </c>
-      <c r="B138" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>overall.noOfParFour</t>
-        </is>
-      </c>
-      <c r="B139" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>overall.parFourTotalStrokes</t>
-        </is>
-      </c>
-      <c r="B140" t="n">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>overall.noOfParFive</t>
-        </is>
-      </c>
-      <c r="B141" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>overall.parFiveTotalStrokes</t>
-        </is>
-      </c>
-      <c r="B142" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>overall.noOfHoles</t>
-        </is>
-      </c>
-      <c r="B143" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>overall.userHcp</t>
-        </is>
-      </c>
-      <c r="B144" t="n">
-        <v>-20.41</v>
       </c>
     </row>
   </sheetData>
@@ -10519,8 +9168,10 @@
           <t>chipHcp (Arccos metric) — PRIORITY</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n">
-        <v>-30</v>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -10529,8 +9180,10 @@
           <t>sandHcp (Arccos metric) — PRIORITY</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n">
-        <v>-4.95</v>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -10551,8 +9204,10 @@
           <t>Chip/short-game save % — PRIORITY</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n">
-        <v>0</v>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -10561,8 +9216,10 @@
           <t>Chip 'get it close' % — PRIORITY</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>11.1</v>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -10571,8 +9228,10 @@
           <t>Chip error rate % — PRIORITY</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n">
-        <v>18.2</v>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -10581,8 +9240,10 @@
           <t>Sand save % — PRIORITY</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n">
-        <v>0</v>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -10591,8 +9252,10 @@
           <t>GIR % (career)</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>27.8</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -10601,8 +9264,10 @@
           <t>Fairway % (career)</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>64.3</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -10611,8 +9276,10 @@
           <t>3-putt % (career)</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>16.7</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -10621,8 +9288,10 @@
           <t>1-putt % (career)</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>5.6</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -10631,8 +9300,10 @@
           <t>Putts / round (career)</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>38</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -10659,7 +9330,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Date pulled: 2026-06-06 23:55 UTC  |  Rounds: 1  Shots: 95</t>
+          <t>Date pulled: 2026-06-07 12:00 UTC  |  Rounds: 1  Shots: 95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
arccos update 2026-06-11, 1 rounds
</commit_message>
<xml_diff>
--- a/arccos_sg_baseline.xlsx
+++ b/arccos_sg_baseline.xlsx
@@ -2868,7 +2868,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6 Iron</t>
+          <t>7 Iron</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8 Iron</t>
+          <t>9 Iron</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>5 Iron</t>
+          <t>6 Iron</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>5 Iron</t>
+          <t>6 Iron</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -5145,12 +5145,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>9 Iron</t>
+          <t>Pitching Wedge</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Wedge</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -5214,12 +5214,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>9 Iron</t>
+          <t>Pitching Wedge</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Wedge</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>7 Iron</t>
+          <t>8 Iron</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>6 Iron</t>
+          <t>7 Iron</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -7836,7 +7836,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -7905,12 +7905,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>9 Iron</t>
+          <t>Pitching Wedge</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Wedge</t>
         </is>
       </c>
       <c r="G76" t="n">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>6 Iron</t>
+          <t>7 Iron</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>8 Iron</t>
+          <t>9 Iron</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -8802,7 +8802,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>6 Iron</t>
+          <t>7 Iron</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -9620,7 +9620,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6 Iron</t>
+          <t>7 Iron</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9676,7 +9676,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5 Iron</t>
+          <t>6 Iron</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9716,7 +9716,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7 Iron</t>
+          <t>8 Iron</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9758,7 +9758,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4 Iron</t>
+          <t>5 Iron</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9812,7 +9812,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8 Iron</t>
+          <t>9 Iron</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9854,12 +9854,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9 Iron</t>
+          <t>Pitching Wedge</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Wedge</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -9904,7 +9904,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>50 Wedge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9958,7 +9958,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>54 Wedge</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9996,7 +9996,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wedge</t>
+          <t>58 Wedge</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -11943,7 +11943,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Date pulled: 2026-06-11 12:00 UTC  |  Rounds: 1  Shots: 95</t>
+          <t>Date pulled: 2026-06-11 23:42 UTC  |  Rounds: 1  Shots: 95</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weather: backfill round weather (temp/wind/dir) from Open-Meteo for both rounds
Arccos carries no weather; populated via Open-Meteo historical archive by course
lat/lng + round mid-time. Enables the wind-correlation analysis the desktop
project flagged as data-gated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arccos_sg_baseline.xlsx
+++ b/arccos_sg_baseline.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT3"/>
+  <dimension ref="A1:AY3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -494,6 +494,11 @@
     <col width="10" customWidth="1" min="44" max="44"/>
     <col width="10" customWidth="1" min="45" max="45"/>
     <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="10" customWidth="1" min="47" max="47"/>
+    <col width="10" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="10" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -727,6 +732,31 @@
           <t>putt_hcp</t>
         </is>
       </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>temp_f</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>wind_mph</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>wind_dir_deg</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>wind_dir</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -875,6 +905,25 @@
       <c r="AT2" t="n">
         <v>-10.2852</v>
       </c>
+      <c r="AU2" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>109</v>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>Drizzle</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1022,6 +1071,25 @@
       </c>
       <c r="AT3" t="n">
         <v>-8.83972</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>129</v>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>Drizzle</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -20274,7 +20342,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Date pulled: 2026-06-14 18:21 UTC  |  Rounds: 2  Shots: 189</t>
+          <t>Date pulled: 2026-06-14 21:32 UTC  |  Rounds: 2  Shots: 189</t>
         </is>
       </c>
     </row>

</xml_diff>